<commit_message>
suport value query in map processor
</commit_message>
<xml_diff>
--- a/test/res/item.xlsx
+++ b/test/res/item.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74214BCD-FD31-4D39-880C-125109FE0FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A30C0F-C3FA-654C-B353-886F4758FAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-15" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="2" r:id="rId1"/>
     <sheet name="item" sheetId="1" r:id="rId2"/>
     <sheet name="follow" sheetId="3" r:id="rId3"/>
     <sheet name="map" sheetId="5" r:id="rId4"/>
-    <sheet name="none" sheetId="4" r:id="rId5"/>
+    <sheet name="map_obj" sheetId="7" r:id="rId5"/>
+    <sheet name="map_arr" sheetId="8" r:id="rId6"/>
+    <sheet name="map_field" sheetId="6" r:id="rId7"/>
+    <sheet name="none" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">define!$A$2:$G$13</definedName>
@@ -109,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="116">
   <si>
     <t>id</t>
   </si>
@@ -457,37 +460,45 @@
     <t>测试22</t>
   </si>
   <si>
-    <t>@map(kind,level)</t>
-    <phoneticPr fontId="8" type="noConversion"/>
-  </si>
-  <si>
     <t>@define</t>
     <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>@map(*,kind,level)</t>
+  </si>
+  <si>
+    <t>@map({name,level,kind},kind,level)</t>
+  </si>
+  <si>
+    <t>@map([name,level],kind,level)</t>
+  </si>
+  <si>
+    <t>@map(.comment,kind,level)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -521,13 +532,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -535,7 +546,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -726,14 +737,35 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1039,30 +1071,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" customWidth="1"/>
-    <col min="3" max="3" width="24.125" customWidth="1"/>
-    <col min="4" max="4" width="21.125" customWidth="1"/>
-    <col min="5" max="5" width="20.375" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.1640625" customWidth="1"/>
+    <col min="4" max="4" width="21.1640625" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
     <col min="6" max="6" width="8.5" customWidth="1"/>
-    <col min="7" max="7" width="9.625" customWidth="1"/>
-    <col min="8" max="8" width="18.375" style="16" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
+      <c r="A1" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+    </row>
+    <row r="2" spans="1:8" ht="16">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1088,7 +1120,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="16">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -1114,7 +1146,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="16">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1126,7 +1158,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="16">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1152,7 +1184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="16">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1168,7 +1200,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="16">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -1188,7 +1220,7 @@
       </c>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="16">
       <c r="A8" s="1" t="s">
         <v>65</v>
       </c>
@@ -1214,7 +1246,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="16">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -1236,7 +1268,7 @@
       </c>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="16">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1258,7 +1290,7 @@
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="16">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1280,7 +1312,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="16">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -1306,7 +1338,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="16">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -1330,7 +1362,7 @@
       </c>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="16">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -1354,7 +1386,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="16">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -1376,7 +1408,7 @@
       </c>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="16">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -1398,7 +1430,7 @@
       </c>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="16">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
@@ -1420,7 +1452,7 @@
       </c>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="16">
       <c r="A18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1455,22 +1487,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="6.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="13.125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="90.875" style="10" customWidth="1"/>
-    <col min="10" max="10" width="24.375" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="90.83203125" style="10" customWidth="1"/>
+    <col min="10" max="10" width="24.33203125" style="10" customWidth="1"/>
     <col min="11" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1502,7 +1534,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1534,7 +1566,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1552,7 +1584,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1584,7 +1616,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="34">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1616,7 +1648,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="4">
         <v>10101</v>
       </c>
@@ -1648,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="4">
         <v>10102</v>
       </c>
@@ -1680,7 +1712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="4">
         <v>10103</v>
       </c>
@@ -1712,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="4">
         <v>10104</v>
       </c>
@@ -1744,7 +1776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="4">
         <v>10105</v>
       </c>
@@ -1776,7 +1808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="4">
         <v>10201</v>
       </c>
@@ -1806,7 +1838,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="4">
         <v>10202</v>
       </c>
@@ -1836,7 +1868,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="4">
         <v>10203</v>
       </c>
@@ -1869,7 +1901,7 @@
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="75"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1880,13 +1912,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B4D15F-7CDD-ED40-889B-A4868E886B80}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" style="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1897,7 +1929,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="16">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1908,14 +1940,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="22"/>
     </row>
-    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="16">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1926,7 +1958,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="17">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1935,7 +1967,7 @@
       </c>
       <c r="C5" s="22"/>
     </row>
-    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="16">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1946,7 +1978,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="16">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -1957,7 +1989,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="16">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1968,7 +2000,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="16">
       <c r="A9" s="4">
         <v>4</v>
       </c>
@@ -1979,14 +2011,14 @@
         <v>97</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" ht="16">
       <c r="A10" s="4">
         <v>5</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="21"/>
     </row>
-    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="16">
       <c r="A11" s="4">
         <v>6</v>
       </c>
@@ -1997,7 +2029,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="16">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -2008,7 +2040,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="16">
       <c r="A13" s="4">
         <v>8</v>
       </c>
@@ -2022,7 +2054,7 @@
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A1:A13">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2031,19 +2063,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E27B46D-4699-4B1C-B2B1-8A327D06725E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" s="27" customFormat="1">
       <c r="A1" s="28" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2060,7 +2092,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>104</v>
       </c>
@@ -2077,7 +2109,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2088,7 +2120,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2105,7 +2137,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2118,7 +2150,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="16">
       <c r="A7" s="25" t="s">
         <v>105</v>
       </c>
@@ -2135,7 +2167,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="16">
       <c r="A8" s="25" t="s">
         <v>105</v>
       </c>
@@ -2152,7 +2184,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="16">
       <c r="A9" s="25" t="s">
         <v>105</v>
       </c>
@@ -2169,7 +2201,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="16">
       <c r="A10" s="25" t="s">
         <v>105</v>
       </c>
@@ -2180,7 +2212,7 @@
         <v>2</v>
       </c>
       <c r="D10" s="26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>110</v>
@@ -2188,6 +2220,338 @@
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="A2:A10">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E541871-473E-3747-A4FF-7005DDAE5E45}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.5" customWidth="1"/>
+    <col min="2" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="27" customFormat="1">
+      <c r="A1" s="28" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16">
+      <c r="A3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="16">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16">
+      <c r="A7" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16">
+      <c r="A8" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="26">
+        <v>1</v>
+      </c>
+      <c r="D8" s="26">
+        <v>2</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16">
+      <c r="A9" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="26">
+        <v>2</v>
+      </c>
+      <c r="D9" s="26">
+        <v>1</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16">
+      <c r="A10" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="26">
+        <v>2</v>
+      </c>
+      <c r="D10" s="26">
+        <v>2</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A10">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D10B9FB-C914-9E4D-9ED5-4AA283A47ADC}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.5" customWidth="1"/>
+    <col min="2" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="27" customFormat="1">
+      <c r="A1" s="28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16">
+      <c r="A3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="16">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16">
+      <c r="A7" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16">
+      <c r="A8" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="26">
+        <v>1</v>
+      </c>
+      <c r="D8" s="26">
+        <v>2</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16">
+      <c r="A9" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="26">
+        <v>2</v>
+      </c>
+      <c r="D9" s="26">
+        <v>1</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16">
+      <c r="A10" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="26">
+        <v>2</v>
+      </c>
+      <c r="D10" s="26">
+        <v>2</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
   <conditionalFormatting sqref="A2:A10">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -2195,12 +2559,178 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA9512F-15D7-C04B-B65B-D43362DB2865}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.5" customWidth="1"/>
+    <col min="2" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="27" customFormat="1">
+      <c r="A1" s="28" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16">
+      <c r="A3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="16">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16">
+      <c r="A7" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16">
+      <c r="A8" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="26">
+        <v>1</v>
+      </c>
+      <c r="D8" s="26">
+        <v>2</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16">
+      <c r="A9" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="26">
+        <v>2</v>
+      </c>
+      <c r="D9" s="26">
+        <v>1</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16">
+      <c r="A10" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="26">
+        <v>2</v>
+      </c>
+      <c r="D10" s="26">
+        <v>2</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A2:A10">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBB972E-C927-480C-A467-3665FD9F033A}">
   <dimension ref="B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2">
       <c r="B2" s="24" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
auto register enum type
</commit_message>
<xml_diff>
--- a/test/res/item.xlsx
+++ b/test/res/item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A30C0F-C3FA-654C-B353-886F4758FAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD7722-8747-4444-861D-0F5876A3A679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37740" yWindow="435" windowWidth="33675" windowHeight="19725" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="2" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
   <si>
     <t>id</t>
   </si>
@@ -401,9 +401,6 @@
     <t>QualityType</t>
   </si>
   <si>
-    <t>bag_type</t>
-  </si>
-  <si>
     <t>物品类型</t>
   </si>
   <si>
@@ -474,31 +471,39 @@
   </si>
   <si>
     <t>@map(.comment,kind,level)</t>
+  </si>
+  <si>
+    <t>ItemType</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>BagType</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -532,13 +537,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -546,7 +551,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -741,7 +746,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
   <dxfs count="6">
@@ -1071,20 +1076,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.1640625" customWidth="1"/>
-    <col min="4" max="4" width="21.1640625" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.875" customWidth="1"/>
+    <col min="3" max="3" width="24.125" customWidth="1"/>
+    <col min="4" max="4" width="21.125" customWidth="1"/>
+    <col min="5" max="5" width="20.375" customWidth="1"/>
     <col min="6" max="6" width="8.5" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="9.625" customWidth="1"/>
+    <col min="8" max="8" width="18.375" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -1094,7 +1099,7 @@
       <c r="G1" s="30"/>
       <c r="H1" s="30"/>
     </row>
-    <row r="2" spans="1:8" ht="16">
+    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1120,7 +1125,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16">
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -1146,7 +1151,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16">
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1158,7 +1163,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" ht="16">
+    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1184,7 +1189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16">
+    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1200,7 +1205,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="16">
+    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -1220,7 +1225,7 @@
       </c>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:8" ht="16">
+    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>65</v>
       </c>
@@ -1243,10 +1248,10 @@
         <v>11</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="16">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -1268,7 +1273,7 @@
       </c>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" ht="16">
+    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1290,7 +1295,7 @@
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="16">
+    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1312,7 +1317,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="16">
+    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -1335,10 +1340,10 @@
         <v>11</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="16">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -1362,7 +1367,7 @@
       </c>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" ht="16">
+    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -1386,7 +1391,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16">
+    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -1408,7 +1413,7 @@
       </c>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="1:8" ht="16">
+    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -1430,7 +1435,7 @@
       </c>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="1:8" ht="16">
+    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
@@ -1452,7 +1457,7 @@
       </c>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="1:8" ht="16">
+    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1487,22 +1492,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="90.83203125" style="10" customWidth="1"/>
-    <col min="10" max="10" width="24.33203125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="32.375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="10" customWidth="1"/>
+    <col min="7" max="7" width="13.125" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="90.875" style="10" customWidth="1"/>
+    <col min="10" max="10" width="24.375" style="10" customWidth="1"/>
     <col min="11" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1534,7 +1539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1548,16 +1553,16 @@
         <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>4</v>
+        <v>73</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="11" t="s">
-        <v>7</v>
+      <c r="H2" s="20" t="s">
+        <v>94</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>14</v>
@@ -1566,7 +1571,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1584,7 +1589,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1616,7 +1621,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="34">
+    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1648,7 +1653,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>10101</v>
       </c>
@@ -1680,7 +1685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>10102</v>
       </c>
@@ -1712,7 +1717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>10103</v>
       </c>
@@ -1744,7 +1749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>10104</v>
       </c>
@@ -1776,7 +1781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>10105</v>
       </c>
@@ -1808,7 +1813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>10201</v>
       </c>
@@ -1838,7 +1843,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>10202</v>
       </c>
@@ -1868,7 +1873,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>10203</v>
       </c>
@@ -1912,13 +1917,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B4D15F-7CDD-ED40-889B-A4868E886B80}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.125" style="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16">
+    <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1929,7 +1934,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16">
+    <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1940,14 +1945,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16">
+    <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="22"/>
     </row>
-    <row r="4" spans="1:3" ht="16">
+    <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1955,19 +1960,19 @@
         <v>10</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="17">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="22"/>
     </row>
-    <row r="6" spans="1:3" ht="16">
+    <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1975,10 +1980,10 @@
         <v>71</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -1986,10 +1991,10 @@
         <v>71</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1997,10 +2002,10 @@
         <v>71</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>4</v>
       </c>
@@ -2008,17 +2013,17 @@
         <v>71</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>5</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="21"/>
     </row>
-    <row r="11" spans="1:3" ht="16">
+    <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>6</v>
       </c>
@@ -2026,10 +2031,10 @@
         <v>74</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -2037,10 +2042,10 @@
         <v>74</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="16">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>8</v>
       </c>
@@ -2048,7 +2053,7 @@
         <v>74</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2063,19 +2068,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E27B46D-4699-4B1C-B2B1-8A327D06725E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
+    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2083,33 +2088,33 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2120,7 +2125,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2128,16 +2133,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2150,29 +2155,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16">
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C8" s="26">
         <v>1</v>
@@ -2181,15 +2186,15 @@
         <v>2</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C9" s="26">
         <v>2</v>
@@ -2198,15 +2203,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C10" s="26">
         <v>2</v>
@@ -2215,7 +2220,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2230,19 +2235,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E541871-473E-3747-A4FF-7005DDAE5E45}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
+    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2250,33 +2255,33 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2287,7 +2292,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2295,16 +2300,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2317,29 +2322,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16">
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C8" s="26">
         <v>1</v>
@@ -2348,15 +2353,15 @@
         <v>2</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C9" s="26">
         <v>2</v>
@@ -2365,15 +2370,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C10" s="26">
         <v>2</v>
@@ -2382,12 +2387,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2396,19 +2402,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D10B9FB-C914-9E4D-9ED5-4AA283A47ADC}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
+    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2416,33 +2422,33 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2453,7 +2459,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2461,16 +2467,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2483,29 +2489,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16">
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C8" s="26">
         <v>1</v>
@@ -2514,15 +2520,15 @@
         <v>2</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C9" s="26">
         <v>2</v>
@@ -2531,15 +2537,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C10" s="26">
         <v>2</v>
@@ -2548,12 +2554,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2562,19 +2569,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA9512F-15D7-C04B-B65B-D43362DB2865}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
+    <row r="1" spans="1:5" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2582,33 +2589,33 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2619,7 +2626,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2627,16 +2634,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2649,29 +2656,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="26">
+        <v>1</v>
+      </c>
+      <c r="D7" s="26">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16">
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C8" s="26">
         <v>1</v>
@@ -2680,15 +2687,15 @@
         <v>2</v>
       </c>
       <c r="E8" s="25" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="16">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C9" s="26">
         <v>2</v>
@@ -2697,15 +2704,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="16">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="25" t="s">
         <v>105</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>106</v>
       </c>
       <c r="C10" s="26">
         <v>2</v>
@@ -2714,12 +2721,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2728,11 +2736,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBB972E-C927-480C-A467-3665FD9F033A}">
   <dimension ref="B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use '$$' to get row data in expr checker
</commit_message>
<xml_diff>
--- a/test/res/item.xlsx
+++ b/test/res/item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF113DD3-916C-AD43-A82F-1A0D070E0E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E13251E-55ED-44B9-A65E-8ECF2B42EF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30780" yWindow="1335" windowWidth="28395" windowHeight="18750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="2" r:id="rId1"/>
@@ -112,7 +112,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="124">
   <si>
     <t>id</t>
   </si>
@@ -408,57 +408,57 @@
   </si>
   <si>
     <t>!@follow(name)</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>s</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>kind</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>level</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>int</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>x</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>auto</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>-</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>测试</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>测试1</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>测试2</t>
   </si>
   <si>
     <t>测试21</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>测试22</t>
   </si>
   <si>
     <t>@define</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>@map(*,kind,level)</t>
@@ -474,42 +474,55 @@
   </si>
   <si>
     <t>ItemType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>BagType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
     <t>@value_type</t>
   </si>
   <si>
     <t>--</t>
+  </si>
+  <si>
+    <t>arr1</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>arr2</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>int[]?</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>[1,2]</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>$.length == arr1.length</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -543,13 +556,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -557,7 +570,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -666,93 +679,88 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
   <dxfs count="6">
@@ -1082,30 +1090,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.1640625" customWidth="1"/>
-    <col min="4" max="4" width="21.1640625" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.875" customWidth="1"/>
+    <col min="3" max="3" width="24.125" customWidth="1"/>
+    <col min="4" max="4" width="21.125" customWidth="1"/>
+    <col min="5" max="5" width="20.375" customWidth="1"/>
     <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="9.625" customWidth="1"/>
+    <col min="8" max="8" width="18.375" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-    </row>
-    <row r="2" spans="1:8" ht="16">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+    </row>
+    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1131,7 +1139,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16">
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -1157,7 +1165,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16">
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1169,7 +1177,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:8" ht="16">
+    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1195,7 +1203,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16">
+    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
@@ -1211,7 +1219,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="16">
+    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>65</v>
       </c>
@@ -1231,7 +1239,7 @@
       </c>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="1:8" ht="16">
+    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>65</v>
       </c>
@@ -1257,7 +1265,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16">
+    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>65</v>
       </c>
@@ -1279,7 +1287,7 @@
       </c>
       <c r="H9" s="18"/>
     </row>
-    <row r="10" spans="1:8" ht="16">
+    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1301,7 +1309,7 @@
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="16">
+    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>65</v>
       </c>
@@ -1323,7 +1331,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="16">
+    <row r="12" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>65</v>
       </c>
@@ -1349,7 +1357,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16">
+    <row r="13" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>65</v>
       </c>
@@ -1373,7 +1381,7 @@
       </c>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" ht="16">
+    <row r="14" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -1397,7 +1405,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16">
+    <row r="15" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -1419,7 +1427,7 @@
       </c>
       <c r="H15" s="19"/>
     </row>
-    <row r="16" spans="1:8" ht="16">
+    <row r="16" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -1441,7 +1449,7 @@
       </c>
       <c r="H16" s="19"/>
     </row>
-    <row r="17" spans="1:8" ht="16">
+    <row r="17" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
@@ -1463,7 +1471,7 @@
       </c>
       <c r="H17" s="19"/>
     </row>
-    <row r="18" spans="1:8" ht="16">
+    <row r="18" spans="1:8" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>65</v>
       </c>
@@ -1489,7 +1497,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -1498,22 +1506,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="32.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="90.83203125" style="10" customWidth="1"/>
-    <col min="10" max="10" width="24.33203125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="5.625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="32.375" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.875" style="10" customWidth="1"/>
+    <col min="7" max="7" width="13.125" style="10" customWidth="1"/>
+    <col min="8" max="8" width="11.625" style="10" customWidth="1"/>
+    <col min="9" max="9" width="90.875" style="10" customWidth="1"/>
+    <col min="10" max="10" width="24.375" style="10" customWidth="1"/>
     <col min="11" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1545,7 +1553,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -1577,7 +1585,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -1595,7 +1603,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1627,7 +1635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="34">
+    <row r="5" spans="1:10" ht="33" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
@@ -1659,7 +1667,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>10101</v>
       </c>
@@ -1691,7 +1699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>10102</v>
       </c>
@@ -1723,7 +1731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>10103</v>
       </c>
@@ -1755,7 +1763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>10104</v>
       </c>
@@ -1787,7 +1795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>10105</v>
       </c>
@@ -1819,7 +1827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>10201</v>
       </c>
@@ -1849,7 +1857,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>10202</v>
       </c>
@@ -1879,7 +1887,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>10203</v>
       </c>
@@ -1910,7 +1918,7 @@
       <c r="J13" s="6"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="5" priority="75"/>
   </conditionalFormatting>
@@ -1922,63 +1930,86 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B4D15F-7CDD-ED40-889B-A4868E886B80}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16">
+    <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="16">
+      <c r="D1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="16">
+      <c r="D2" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="22"/>
-    </row>
-    <row r="4" spans="1:3" ht="16">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="17">
+      <c r="D4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="22"/>
-    </row>
-    <row r="6" spans="1:3" ht="16">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1988,8 +2019,14 @@
       <c r="C6" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="16">
+      <c r="D6" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -1999,8 +2036,10 @@
       <c r="C7" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="16">
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -2010,8 +2049,10 @@
       <c r="C8" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="16">
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>4</v>
       </c>
@@ -2021,15 +2062,19 @@
       <c r="C9" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="16">
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>5</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="21"/>
-    </row>
-    <row r="11" spans="1:3" ht="16">
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>6</v>
       </c>
@@ -2039,8 +2084,10 @@
       <c r="C11" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="16">
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -2050,8 +2097,10 @@
       <c r="C12" s="21" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="16">
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+    </row>
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>8</v>
       </c>
@@ -2061,9 +2110,11 @@
       <c r="C13" s="21" t="s">
         <v>96</v>
       </c>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A1:A13">
     <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
@@ -2074,19 +2125,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E27B46D-4699-4B1C-B2B1-8A327D06725E}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>118</v>
       </c>
@@ -2103,7 +2154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2120,7 +2171,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2131,7 +2182,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2148,7 +2199,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2161,76 +2212,76 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="24">
+        <v>1</v>
+      </c>
+      <c r="D7" s="24">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="26">
-        <v>1</v>
-      </c>
-      <c r="D8" s="26">
+      <c r="C8" s="24">
+        <v>1</v>
+      </c>
+      <c r="D8" s="24">
         <v>2</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16">
-      <c r="A9" s="25" t="s">
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="24">
         <v>2</v>
       </c>
-      <c r="D9" s="26">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="s">
+      <c r="D9" s="24">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="24">
         <v>2</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="24">
         <v>2</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="23" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
@@ -2241,19 +2292,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E541871-473E-3747-A4FF-7005DDAE5E45}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2270,7 +2321,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2287,7 +2338,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2298,7 +2349,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2315,7 +2366,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2328,76 +2379,76 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="24">
+        <v>1</v>
+      </c>
+      <c r="D7" s="24">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="26">
-        <v>1</v>
-      </c>
-      <c r="D8" s="26">
+      <c r="C8" s="24">
+        <v>1</v>
+      </c>
+      <c r="D8" s="24">
         <v>2</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16">
-      <c r="A9" s="25" t="s">
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="24">
         <v>2</v>
       </c>
-      <c r="D9" s="26">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="s">
+      <c r="D9" s="24">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="24">
         <v>2</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="24">
         <v>2</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="23" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
@@ -2408,19 +2459,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D10B9FB-C914-9E4D-9ED5-4AA283A47ADC}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2437,7 +2488,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2454,7 +2505,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2465,7 +2516,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2482,7 +2533,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2495,76 +2546,76 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="24">
+        <v>1</v>
+      </c>
+      <c r="D7" s="24">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="26">
-        <v>1</v>
-      </c>
-      <c r="D8" s="26">
+      <c r="C8" s="24">
+        <v>1</v>
+      </c>
+      <c r="D8" s="24">
         <v>2</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16">
-      <c r="A9" s="25" t="s">
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="24">
         <v>2</v>
       </c>
-      <c r="D9" s="26">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="s">
+      <c r="D9" s="24">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="24">
         <v>2</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="24">
         <v>2</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="23" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
@@ -2575,19 +2626,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA9512F-15D7-C04B-B65B-D43362DB2865}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="27" customFormat="1">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2604,7 +2655,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>103</v>
       </c>
@@ -2621,7 +2672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2632,7 +2683,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -2649,7 +2700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
@@ -2662,76 +2713,76 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="26">
-        <v>1</v>
-      </c>
-      <c r="D7" s="26">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="s">
+      <c r="C7" s="24">
+        <v>1</v>
+      </c>
+      <c r="D7" s="24">
+        <v>1</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="26">
-        <v>1</v>
-      </c>
-      <c r="D8" s="26">
+      <c r="C8" s="24">
+        <v>1</v>
+      </c>
+      <c r="D8" s="24">
         <v>2</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="23" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="16">
-      <c r="A9" s="25" t="s">
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="24">
         <v>2</v>
       </c>
-      <c r="D9" s="26">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="s">
+      <c r="D9" s="24">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="16">
-      <c r="A10" s="25" t="s">
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="24">
         <v>2</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="24">
         <v>2</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="23" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="A2:A10">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -2742,15 +2793,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADBB972E-C927-480C-A467-3665FD9F033A}">
   <dimension ref="B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:2">
-      <c r="B2" s="24" t="s">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B2" s="22" t="s">
         <v>98</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>